<commit_message>
scan: seg4 2026-07-10 17:48 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq5_2026-07-09.xlsx
+++ b/output/full_scan/batch_seq5_2026-07-09.xlsx
@@ -9707,7 +9707,7 @@
         <v/>
       </c>
       <c r="D175" s="2" t="n">
-        <v>369.4932262641656</v>
+        <v>369.4932262641694</v>
       </c>
       <c r="E175" s="2" t="n">
         <v>30</v>
@@ -9721,10 +9721,10 @@
         <v>0</v>
       </c>
       <c r="H175" s="2" t="n">
-        <v>47.50974289300732</v>
+        <v>47.50974292287961</v>
       </c>
       <c r="I175" s="2" t="n">
-        <v>22.46633967890924</v>
+        <v>22.46633972719823</v>
       </c>
       <c r="J175" s="2" t="n">
         <v>0.4600528172509878</v>
@@ -9739,7 +9739,7 @@
         <v>-1</v>
       </c>
       <c r="N175" s="2" t="n">
-        <v>0.0448590279386785</v>
+        <v>0.0448590274807738</v>
       </c>
       <c r="O175" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
scan: seg4 2026-07-10 20:12 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq5_2026-07-09.xlsx
+++ b/output/full_scan/batch_seq5_2026-07-09.xlsx
@@ -1693,21 +1693,21 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>5487</v>
+        <v>6121</v>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>通泰</t>
+          <t>新普</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
         <v/>
       </c>
       <c r="D24" s="2" t="n">
-        <v>767.8153561370052</v>
+        <v>768.2195400059876</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>28.7</v>
+        <v>420.5</v>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
@@ -1718,49 +1718,49 @@
         <v>0</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>53.43111090844679</v>
+        <v>51.03227246071479</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>33.95660232411846</v>
+        <v>27.22275383125953</v>
       </c>
       <c r="J24" s="2" t="n">
-        <v>1.519766346118588</v>
+        <v>0.8908416609528386</v>
       </c>
       <c r="K24" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L24" s="2" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="M24" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>0.0274441222090457</v>
+        <v>0.4387885186075202</v>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, kd_golden_cross, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, invest_trust_buy_2d, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>4973</v>
+        <v>5487</v>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>廣穎</t>
+          <t>通泰</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
         <v/>
       </c>
       <c r="D25" s="2" t="n">
-        <v>765.8311331052814</v>
+        <v>767.8153561370052</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>166.5</v>
+        <v>28.7</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
@@ -1771,16 +1771,16 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>50.31848131709806</v>
+        <v>53.43111090844679</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>26.38621011815188</v>
+        <v>33.95660232411846</v>
       </c>
       <c r="J25" s="2" t="n">
-        <v>0.7620383488812934</v>
+        <v>1.519766346118588</v>
       </c>
       <c r="K25" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L25" s="2" t="n">
         <v>0</v>
@@ -1789,31 +1789,31 @@
         <v>-1</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>-4.60603940110569</v>
+        <v>0.0274441222090457</v>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, stronger_than_market, kd_golden_cross, above_ichimoku_cloud</t>
+          <t>volume_break, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, kd_golden_cross, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>5371</v>
+        <v>4973</v>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>中光電</t>
+          <t>廣穎</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
         <v/>
       </c>
       <c r="D26" s="2" t="n">
-        <v>763.1811176132519</v>
+        <v>765.8311331052814</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>93.2</v>
+        <v>166.5</v>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
@@ -1824,16 +1824,16 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>60.85775701927957</v>
+        <v>50.31848131709806</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>29.49073301285372</v>
+        <v>26.38621011815188</v>
       </c>
       <c r="J26" s="2" t="n">
-        <v>2.474611775870327</v>
+        <v>0.7620383488812934</v>
       </c>
       <c r="K26" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L26" s="2" t="n">
         <v>0</v>
@@ -1842,31 +1842,31 @@
         <v>-1</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>1.918602538518536</v>
+        <v>-4.60603940110569</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>volume_break, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, stronger_than_market, kd_golden_cross, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>6109</v>
+        <v>5371</v>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>亞元</t>
+          <t>中光電</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
         <v/>
       </c>
       <c r="D27" s="2" t="n">
-        <v>762.3263453816904</v>
+        <v>763.1811176132519</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>13.1</v>
+        <v>93.2</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
@@ -1877,13 +1877,13 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>55.63178388840297</v>
+        <v>60.85775701927957</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>32.84610747033704</v>
+        <v>29.49073301285372</v>
       </c>
       <c r="J27" s="2" t="n">
-        <v>0.5450410013211663</v>
+        <v>2.474611775870327</v>
       </c>
       <c r="K27" s="2" t="n">
         <v>0</v>
@@ -1895,31 +1895,31 @@
         <v>-1</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>0.0546811097215454</v>
+        <v>1.918602538518536</v>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>volume_break, rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>5489</v>
+        <v>6109</v>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>彩富</t>
+          <t>亞元</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
         <v/>
       </c>
       <c r="D28" s="2" t="n">
-        <v>762.1639138451682</v>
+        <v>762.3263453816904</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>61.7</v>
+        <v>13.1</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
@@ -1930,13 +1930,13 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>61.55147021212415</v>
+        <v>55.63178388840297</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>47.96277321021014</v>
+        <v>32.84610747033704</v>
       </c>
       <c r="J28" s="2" t="n">
-        <v>0.597948049187966</v>
+        <v>0.5450410013211663</v>
       </c>
       <c r="K28" s="2" t="n">
         <v>0</v>
@@ -1948,7 +1948,7 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>0.2235861322515919</v>
+        <v>0.0546811097215454</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
@@ -1958,21 +1958,21 @@
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>6103</v>
+        <v>5489</v>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>合邦</t>
+          <t>彩富</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
         <v/>
       </c>
       <c r="D29" s="2" t="n">
-        <v>756.5818050360501</v>
+        <v>762.1639138451682</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>30.6</v>
+        <v>61.7</v>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
@@ -1983,13 +1983,13 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>51.77926771658405</v>
+        <v>61.55147021212415</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>6.731647694547544</v>
+        <v>47.96277321021014</v>
       </c>
       <c r="J29" s="2" t="n">
-        <v>5.19465005652851</v>
+        <v>0.597948049187966</v>
       </c>
       <c r="K29" s="2" t="n">
         <v>0</v>
@@ -2001,31 +2001,31 @@
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>0.6445874460213974</v>
+        <v>0.2235861322515919</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, ema60_gt_ema120, volume_break, market_above_ma60, hist_turn_positive, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>6146</v>
+        <v>6103</v>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>耕興</t>
+          <t>合邦</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
         <v/>
       </c>
       <c r="D30" s="2" t="n">
-        <v>746.8093349845714</v>
+        <v>756.5818050360501</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>206</v>
+        <v>30.6</v>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
@@ -2036,13 +2036,13 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>54.60128894119454</v>
+        <v>51.77926771658405</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>30.3026150641962</v>
+        <v>6.731647694547544</v>
       </c>
       <c r="J30" s="2" t="n">
-        <v>1.168147981564122</v>
+        <v>5.19465005652851</v>
       </c>
       <c r="K30" s="2" t="n">
         <v>0</v>
@@ -2054,31 +2054,31 @@
         <v>-1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>2.515474087258776</v>
+        <v>0.6445874460213974</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, bb_squeeze_breakout, mfi_strong</t>
+          <t>macd_golden_cross, ema60_gt_ema120, volume_break, market_above_ma60, hist_turn_positive, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>6141</v>
+        <v>6146</v>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>柏承</t>
+          <t>耕興</t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
         <v/>
       </c>
       <c r="D31" s="2" t="n">
-        <v>745.3245557506359</v>
+        <v>746.8093349845714</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>39.05</v>
+        <v>206</v>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
@@ -2089,13 +2089,13 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>55.61967467493864</v>
+        <v>54.60128894119454</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>19.36986333297704</v>
+        <v>30.3026150641962</v>
       </c>
       <c r="J31" s="2" t="n">
-        <v>1.149105939182292</v>
+        <v>1.168147981564122</v>
       </c>
       <c r="K31" s="2" t="n">
         <v>0</v>
@@ -2107,31 +2107,31 @@
         <v>-1</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>-0.2112895615338184</v>
+        <v>2.515474087258776</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, obv_uptrend, williams_r_recovery, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, bb_squeeze_breakout, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>6113</v>
+        <v>6141</v>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>亞矽</t>
+          <t>柏承</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
         <v/>
       </c>
       <c r="D32" s="2" t="n">
-        <v>734.9158484229325</v>
+        <v>745.3245557506359</v>
       </c>
       <c r="E32" s="2" t="n">
-        <v>27.7</v>
+        <v>39.05</v>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
@@ -2142,16 +2142,16 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>55.03192761885502</v>
+        <v>55.61967467493864</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>25.18304164759625</v>
+        <v>19.36986333297704</v>
       </c>
       <c r="J32" s="2" t="n">
-        <v>0.8951426128792889</v>
+        <v>1.149105939182292</v>
       </c>
       <c r="K32" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L32" s="2" t="n">
         <v>0</v>
@@ -2160,31 +2160,31 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>-0.2249185379866054</v>
+        <v>-0.2112895615338184</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, obv_uptrend, williams_r_recovery, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>4536</v>
+        <v>6113</v>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>拓凱</t>
+          <t>亞矽</t>
         </is>
       </c>
       <c r="C33" s="2" t="n">
         <v/>
       </c>
       <c r="D33" s="2" t="n">
-        <v>722.2806472490196</v>
+        <v>734.9158484229325</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>171.5</v>
+        <v>27.7</v>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
@@ -2195,16 +2195,16 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>63.40180908759909</v>
+        <v>55.03192761885502</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>27.29433330305982</v>
+        <v>25.18304164759625</v>
       </c>
       <c r="J33" s="2" t="n">
-        <v>0.9627687442768682</v>
+        <v>0.8951426128792889</v>
       </c>
       <c r="K33" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L33" s="2" t="n">
         <v>0</v>
@@ -2213,31 +2213,31 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>0.457501796328835</v>
+        <v>-0.2249185379866054</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>4976</v>
+        <v>4536</v>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>佳凌</t>
+          <t>拓凱</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
         <v/>
       </c>
       <c r="D34" s="2" t="n">
-        <v>712.2195854802842</v>
+        <v>722.2806472490196</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>38.3</v>
+        <v>171.5</v>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
@@ -2248,16 +2248,16 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>53.59040160139187</v>
+        <v>63.40180908759909</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>32.90419022818279</v>
+        <v>27.29433330305982</v>
       </c>
       <c r="J34" s="2" t="n">
-        <v>0.4390687358783951</v>
+        <v>0.9627687442768682</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L34" s="2" t="n">
         <v>0</v>
@@ -2266,31 +2266,31 @@
         <v>-1</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>-0.4039540296353701</v>
+        <v>0.457501796328835</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, kd_golden_cross, obv_uptrend, above_ichimoku_cloud</t>
+          <t>rsi_strong, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>4590</v>
+        <v>4976</v>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>富田-創</t>
+          <t>佳凌</t>
         </is>
       </c>
       <c r="C35" s="2" t="n">
         <v/>
       </c>
       <c r="D35" s="2" t="n">
-        <v>708.8732103981085</v>
+        <v>712.2195854802842</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>90.40000000000001</v>
+        <v>38.3</v>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
@@ -2301,16 +2301,16 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>62.73125699060857</v>
+        <v>53.59040160139187</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>24.88617935380314</v>
+        <v>32.90419022818279</v>
       </c>
       <c r="J35" s="2" t="n">
-        <v>0.965207566965144</v>
+        <v>0.4390687358783951</v>
       </c>
       <c r="K35" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L35" s="2" t="n">
         <v>0</v>
@@ -2319,31 +2319,31 @@
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>1.295972622635541</v>
+        <v>-0.4039540296353701</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, stronger_than_market, kd_golden_cross, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>6129</v>
+        <v>4590</v>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>普誠</t>
+          <t>富田-創</t>
         </is>
       </c>
       <c r="C36" s="2" t="n">
         <v/>
       </c>
       <c r="D36" s="2" t="n">
-        <v>707.2149572583246</v>
+        <v>708.8732103981085</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>19</v>
+        <v>90.40000000000001</v>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
@@ -2354,16 +2354,16 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>56.39539468779272</v>
+        <v>62.73125699060857</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>33.4512709772529</v>
+        <v>24.88617935380314</v>
       </c>
       <c r="J36" s="2" t="n">
-        <v>0.5216115509669587</v>
+        <v>0.965207566965144</v>
       </c>
       <c r="K36" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L36" s="2" t="n">
         <v>0</v>
@@ -2372,31 +2372,31 @@
         <v>-1</v>
       </c>
       <c r="N36" s="2" t="n">
-        <v>0.06341357908675441</v>
+        <v>1.295972622635541</v>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>rsi_strong, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>6138</v>
+        <v>6129</v>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>茂達</t>
+          <t>普誠</t>
         </is>
       </c>
       <c r="C37" s="2" t="n">
         <v/>
       </c>
       <c r="D37" s="2" t="n">
-        <v>704.3352998367152</v>
+        <v>707.2149572583246</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>376</v>
+        <v>19</v>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
@@ -2407,49 +2407,49 @@
         <v>0</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>53.47547853345058</v>
+        <v>56.39539468779272</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>22.26069863618862</v>
+        <v>33.4512709772529</v>
       </c>
       <c r="J37" s="2" t="n">
-        <v>0.9599632317727542</v>
+        <v>0.5216115509669587</v>
       </c>
       <c r="K37" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L37" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="M37" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>-0.2284695436153079</v>
+        <v>0.06341357908675441</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, invest_trust_buy_2d, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, adx_trending, kd_golden_cross, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>6143</v>
+        <v>6138</v>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>振曜</t>
+          <t>茂達</t>
         </is>
       </c>
       <c r="C38" s="2" t="n">
         <v/>
       </c>
       <c r="D38" s="2" t="n">
-        <v>704.2237624723317</v>
+        <v>704.3352998367152</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>104.5</v>
+        <v>376</v>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
@@ -2460,49 +2460,49 @@
         <v>0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>65.07049253566694</v>
+        <v>53.47547853345058</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>26.83535939664905</v>
+        <v>22.26069863618862</v>
       </c>
       <c r="J38" s="2" t="n">
-        <v>0.4670608436982588</v>
+        <v>0.9599632317727542</v>
       </c>
       <c r="K38" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L38" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M38" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>1.750187942902223</v>
+        <v>-0.2284695436153079</v>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, invest_trust_buy_2d, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>6147</v>
+        <v>6143</v>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>頎邦</t>
+          <t>振曜</t>
         </is>
       </c>
       <c r="C39" s="2" t="n">
         <v/>
       </c>
       <c r="D39" s="2" t="n">
-        <v>699.0818577006442</v>
+        <v>704.2237624723317</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>217</v>
+        <v>104.5</v>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
@@ -2513,16 +2513,16 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>47.56179822800908</v>
+        <v>65.07049253566694</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>17.85833652849296</v>
+        <v>26.83535939664905</v>
       </c>
       <c r="J39" s="2" t="n">
-        <v>1.289118791361319</v>
+        <v>0.4670608436982588</v>
       </c>
       <c r="K39" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L39" s="2" t="n">
         <v>0</v>
@@ -2531,31 +2531,31 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>-4.11444709395332</v>
+        <v>1.750187942902223</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, stronger_than_market, kd_golden_cross, obv_uptrend</t>
+          <t>rsi_strong, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>5871</v>
+        <v>6147</v>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>中租-KY</t>
+          <t>頎邦</t>
         </is>
       </c>
       <c r="C40" s="2" t="n">
         <v/>
       </c>
       <c r="D40" s="2" t="n">
-        <v>697.8381425580187</v>
+        <v>699.0818577006442</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>114.5</v>
+        <v>217</v>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
@@ -2566,49 +2566,49 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>48.6488267504171</v>
+        <v>47.56179822800908</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>8.483369611834494</v>
+        <v>17.85833652849296</v>
       </c>
       <c r="J40" s="2" t="n">
-        <v>0.6057245764785334</v>
+        <v>1.289118791361319</v>
       </c>
       <c r="K40" s="2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L40" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M40" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>-0.2769141422948607</v>
+        <v>-4.11444709395332</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, invest_trust_buy_2d, dealer_buy_3d, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, stronger_than_market, kd_golden_cross, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>6139</v>
+        <v>5871</v>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>亞翔</t>
+          <t>中租-KY</t>
         </is>
       </c>
       <c r="C41" s="2" t="n">
         <v/>
       </c>
       <c r="D41" s="2" t="n">
-        <v>692.7861615903009</v>
+        <v>697.8381425580187</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>875</v>
+        <v>114.5</v>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
@@ -2619,49 +2619,49 @@
         <v>0</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>53.69986271090175</v>
+        <v>48.6488267504171</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>23.52410337869207</v>
+        <v>8.483369611834494</v>
       </c>
       <c r="J41" s="2" t="n">
-        <v>0.5888280838123039</v>
+        <v>0.6057245764785334</v>
       </c>
       <c r="K41" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L41" s="2" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="M41" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>-4.551831518437382</v>
+        <v>-0.2769141422948607</v>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, invest_trust_buy_2d, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, invest_trust_buy_2d, dealer_buy_3d, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>4545</v>
+        <v>6139</v>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>銘鈺</t>
+          <t>亞翔</t>
         </is>
       </c>
       <c r="C42" s="2" t="n">
         <v/>
       </c>
       <c r="D42" s="2" t="n">
-        <v>685.506595321879</v>
+        <v>692.7861615903009</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>38.3</v>
+        <v>875</v>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
@@ -2672,49 +2672,49 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>54.933398107528</v>
+        <v>53.69986271090175</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>32.50716632875244</v>
+        <v>23.52410337869207</v>
       </c>
       <c r="J42" s="2" t="n">
-        <v>0.3286675523936056</v>
+        <v>0.5888280838123039</v>
       </c>
       <c r="K42" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L42" s="2" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="M42" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>-0.0864294859690139</v>
+        <v>-4.551831518437382</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, kd_golden_cross, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, invest_trust_buy_2d, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>5328</v>
+        <v>4545</v>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>華容</t>
+          <t>銘鈺</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
         <v/>
       </c>
       <c r="D43" s="2" t="n">
-        <v>683.3322773273171</v>
+        <v>685.506595321879</v>
       </c>
       <c r="E43" s="2" t="n">
-        <v>70.5</v>
+        <v>38.3</v>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
@@ -2725,16 +2725,16 @@
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>61.6225412598008</v>
+        <v>54.933398107528</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>50.53099950758629</v>
+        <v>32.50716632875244</v>
       </c>
       <c r="J43" s="2" t="n">
-        <v>0.5033929752859468</v>
+        <v>0.3286675523936056</v>
       </c>
       <c r="K43" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L43" s="2" t="n">
         <v>0</v>
@@ -2743,31 +2743,31 @@
         <v>-1</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>-0.1407247399826037</v>
+        <v>-0.0864294859690139</v>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, kd_golden_cross, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>4949</v>
+        <v>5328</v>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>有成精密</t>
+          <t>華容</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
         <v/>
       </c>
       <c r="D44" s="2" t="n">
-        <v>678.24320216443</v>
+        <v>683.3322773273171</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>79</v>
+        <v>70.5</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
@@ -2778,16 +2778,16 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>43.57113845646791</v>
+        <v>61.6225412598008</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>23.68820689701126</v>
+        <v>50.53099950758629</v>
       </c>
       <c r="J44" s="2" t="n">
-        <v>0.8820560798211919</v>
+        <v>0.5033929752859468</v>
       </c>
       <c r="K44" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L44" s="2" t="n">
         <v>0</v>
@@ -2796,31 +2796,31 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>-0.6700390797656679</v>
+        <v>-0.1407247399826037</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, stronger_than_market, kd_golden_cross</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>6156</v>
+        <v>4949</v>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>松上</t>
+          <t>有成精密</t>
         </is>
       </c>
       <c r="C45" s="2" t="n">
         <v/>
       </c>
       <c r="D45" s="2" t="n">
-        <v>673.4459943968557</v>
+        <v>678.24320216443</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>26.95</v>
+        <v>79</v>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
@@ -2831,16 +2831,16 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>56.09383595666467</v>
+        <v>43.57113845646791</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>42.68444711644433</v>
+        <v>23.68820689701126</v>
       </c>
       <c r="J45" s="2" t="n">
-        <v>0.3829379372669391</v>
+        <v>0.8820560798211919</v>
       </c>
       <c r="K45" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L45" s="2" t="n">
         <v>0</v>
@@ -2849,31 +2849,31 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>-0.0942718590617746</v>
+        <v>-0.6700390797656679</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, stronger_than_market, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>6152</v>
+        <v>6156</v>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>百一</t>
+          <t>松上</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
         <v/>
       </c>
       <c r="D46" s="2" t="n">
-        <v>672.57541119207</v>
+        <v>673.4459943968557</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>13.45</v>
+        <v>26.95</v>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
@@ -2884,16 +2884,16 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>41.8973511714966</v>
+        <v>56.09383595666467</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>11.76568835069056</v>
+        <v>42.68444711644433</v>
       </c>
       <c r="J46" s="2" t="n">
-        <v>0.6741664422575429</v>
+        <v>0.3829379372669391</v>
       </c>
       <c r="K46" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L46" s="2" t="n">
         <v>0</v>
@@ -2902,31 +2902,31 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>0.0072230797297521</v>
+        <v>-0.0942718590617746</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, ema60_gt_ema120, market_above_ma60, avoid_chase, hist_turn_positive, stronger_than_market, kd_golden_cross, obv_uptrend</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>5475</v>
+        <v>6152</v>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>德宏</t>
+          <t>百一</t>
         </is>
       </c>
       <c r="C47" s="2" t="n">
         <v/>
       </c>
       <c r="D47" s="2" t="n">
-        <v>655.018976921002</v>
+        <v>672.57541119207</v>
       </c>
       <c r="E47" s="2" t="n">
-        <v>192.5</v>
+        <v>13.45</v>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
@@ -2937,49 +2937,49 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>33.78999828369341</v>
+        <v>41.8973511714966</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>20.73780733967266</v>
+        <v>11.76568835069056</v>
       </c>
       <c r="J47" s="2" t="n">
-        <v>1.767999847372974</v>
+        <v>0.6741664422575429</v>
       </c>
       <c r="K47" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L47" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M47" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>-3.545083739783166</v>
+        <v>0.0072230797297521</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, invest_trust_buy_2d</t>
+          <t>macd_golden_cross, ema60_gt_ema120, market_above_ma60, avoid_chase, hist_turn_positive, stronger_than_market, kd_golden_cross, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>4931</v>
+        <v>5475</v>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>新盛力</t>
+          <t>德宏</t>
         </is>
       </c>
       <c r="C48" s="2" t="n">
         <v/>
       </c>
       <c r="D48" s="2" t="n">
-        <v>653.8949041373809</v>
+        <v>655.018976921002</v>
       </c>
       <c r="E48" s="2" t="n">
-        <v>255</v>
+        <v>192.5</v>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
@@ -2990,49 +2990,49 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>54.62396684129079</v>
+        <v>33.78999828369341</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>20.84237015790699</v>
+        <v>20.73780733967266</v>
       </c>
       <c r="J48" s="2" t="n">
-        <v>2.575908757257201</v>
+        <v>1.767999847372974</v>
       </c>
       <c r="K48" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L48" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M48" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>-0.7772662569597912</v>
+        <v>-3.545083739783166</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase, liquidity_ok, foreign_buy_3d, adx_trending, invest_trust_buy_2d</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>5302</v>
+        <v>4931</v>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>太欣</t>
+          <t>新盛力</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
         <v/>
       </c>
       <c r="D49" s="2" t="n">
-        <v>650.5315179333396</v>
+        <v>653.8949041373809</v>
       </c>
       <c r="E49" s="2" t="n">
-        <v>13.25</v>
+        <v>255</v>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
@@ -3043,16 +3043,16 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>53.62930195904802</v>
+        <v>54.62396684129079</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>37.39521693957945</v>
+        <v>20.84237015790699</v>
       </c>
       <c r="J49" s="2" t="n">
-        <v>0.4866092862661319</v>
+        <v>2.575908757257201</v>
       </c>
       <c r="K49" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L49" s="2" t="n">
         <v>0</v>
@@ -3061,31 +3061,31 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>0.0382272072100513</v>
+        <v>-0.7772662569597912</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, volume_break, market_above_ma60, liquidity_ok, adx_trending, stronger_than_market, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>5607</v>
+        <v>5302</v>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>遠雄港</t>
+          <t>太欣</t>
         </is>
       </c>
       <c r="C50" s="2" t="n">
         <v/>
       </c>
       <c r="D50" s="2" t="n">
-        <v>649.2972510271251</v>
+        <v>650.5315179333396</v>
       </c>
       <c r="E50" s="2" t="n">
-        <v>51.4</v>
+        <v>13.25</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
@@ -3096,16 +3096,16 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>52.07619845110473</v>
+        <v>53.62930195904802</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>15.67258524320981</v>
+        <v>37.39521693957945</v>
       </c>
       <c r="J50" s="2" t="n">
-        <v>0.7169028070980746</v>
+        <v>0.4866092862661319</v>
       </c>
       <c r="K50" s="2" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L50" s="2" t="n">
         <v>0</v>
@@ -3114,31 +3114,31 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>-0.059836010935835</v>
+        <v>0.0382272072100513</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, foreign_buy_3d, stronger_than_market, kd_golden_cross, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending, stronger_than_market, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>4938</v>
+        <v>5607</v>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>和碩</t>
+          <t>遠雄港</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
         <v/>
       </c>
       <c r="D51" s="2" t="n">
-        <v>641.6535486174395</v>
+        <v>649.2972510271251</v>
       </c>
       <c r="E51" s="2" t="n">
-        <v>82.7</v>
+        <v>51.4</v>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
@@ -3149,49 +3149,49 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>45.92567820686074</v>
+        <v>52.07619845110473</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>13.0970640914021</v>
+        <v>15.67258524320981</v>
       </c>
       <c r="J51" s="2" t="n">
-        <v>0.2668303914375913</v>
+        <v>0.7169028070980746</v>
       </c>
       <c r="K51" s="2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L51" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M51" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>-0.1553241384524937</v>
+        <v>-0.059836010935835</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, obv_uptrend, dealer_buy_3d, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, foreign_buy_3d, stronger_than_market, kd_golden_cross, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>5481</v>
+        <v>4938</v>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>新華</t>
+          <t>和碩</t>
         </is>
       </c>
       <c r="C52" s="2" t="n">
         <v/>
       </c>
       <c r="D52" s="2" t="n">
-        <v>641.5219664343792</v>
+        <v>641.6535486174395</v>
       </c>
       <c r="E52" s="2" t="n">
-        <v>21</v>
+        <v>82.7</v>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
@@ -3202,49 +3202,49 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>51.97117299352748</v>
+        <v>45.92567820686074</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>22.85023406321423</v>
+        <v>13.0970640914021</v>
       </c>
       <c r="J52" s="2" t="n">
-        <v>1.925781820838813</v>
+        <v>0.2668303914375913</v>
       </c>
       <c r="K52" s="2" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L52" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M52" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>-0.10072122234934</v>
+        <v>-0.1553241384524937</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, stronger_than_market, obv_uptrend, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, stronger_than_market, obv_uptrend, dealer_buy_3d, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>5490</v>
+        <v>5481</v>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>同亨</t>
+          <t>新華</t>
         </is>
       </c>
       <c r="C53" s="2" t="n">
         <v/>
       </c>
       <c r="D53" s="2" t="n">
-        <v>641.3322273292895</v>
+        <v>641.5219664343792</v>
       </c>
       <c r="E53" s="2" t="n">
-        <v>29.95</v>
+        <v>21</v>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
@@ -3255,16 +3255,16 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>55.31911618474639</v>
+        <v>51.97117299352748</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>22.77002389094239</v>
+        <v>22.85023406321423</v>
       </c>
       <c r="J53" s="2" t="n">
-        <v>0.7017658181461784</v>
+        <v>1.925781820838813</v>
       </c>
       <c r="K53" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L53" s="2" t="n">
         <v>0</v>
@@ -3273,31 +3273,31 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>0.1537416252183485</v>
+        <v>-0.10072122234934</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, adx_trending, stronger_than_market, mfi_strong, above_ichimoku_cloud</t>
+          <t>volume_break, market_above_ma60, avoid_chase, foreign_buy_3d, adx_trending, stronger_than_market, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>5344</v>
+        <v>5490</v>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>立衛</t>
+          <t>同亨</t>
         </is>
       </c>
       <c r="C54" s="2" t="n">
         <v/>
       </c>
       <c r="D54" s="2" t="n">
-        <v>640.8616005375287</v>
+        <v>641.3322273292895</v>
       </c>
       <c r="E54" s="2" t="n">
-        <v>16.3</v>
+        <v>29.95</v>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
@@ -3308,16 +3308,16 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>51.42930391611786</v>
+        <v>55.31911618474639</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>17.86089550557363</v>
+        <v>22.77002389094239</v>
       </c>
       <c r="J54" s="2" t="n">
-        <v>0.7430419558253353</v>
+        <v>0.7017658181461784</v>
       </c>
       <c r="K54" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L54" s="2" t="n">
         <v>0</v>
@@ -3326,31 +3326,31 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>0.0657636123556823</v>
+        <v>0.1537416252183485</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, foreign_buy_3d, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, rsi_strong, market_above_ma60, adx_trending, stronger_than_market, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>5388</v>
+        <v>5344</v>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>中磊</t>
+          <t>立衛</t>
         </is>
       </c>
       <c r="C55" s="2" t="n">
         <v/>
       </c>
       <c r="D55" s="2" t="n">
-        <v>640.7135047260184</v>
+        <v>640.8616005375287</v>
       </c>
       <c r="E55" s="2" t="n">
-        <v>84.59999999999999</v>
+        <v>16.3</v>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
@@ -3361,16 +3361,16 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>54.89195528384244</v>
+        <v>51.42930391611786</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>13.84676242588044</v>
+        <v>17.86089550557363</v>
       </c>
       <c r="J55" s="2" t="n">
-        <v>1.701396182975228</v>
+        <v>0.7430419558253353</v>
       </c>
       <c r="K55" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L55" s="2" t="n">
         <v>0</v>
@@ -3379,31 +3379,31 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>0.3910592841563549</v>
+        <v>0.0657636123556823</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, liquidity_ok, stronger_than_market, kd_golden_cross, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, foreign_buy_3d, stronger_than_market, obv_uptrend, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>6155</v>
+        <v>5388</v>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>鈞寶</t>
+          <t>中磊</t>
         </is>
       </c>
       <c r="C56" s="2" t="n">
         <v/>
       </c>
       <c r="D56" s="2" t="n">
-        <v>629.4959232885302</v>
+        <v>640.7135047260184</v>
       </c>
       <c r="E56" s="2" t="n">
-        <v>73.2</v>
+        <v>84.59999999999999</v>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
@@ -3414,16 +3414,16 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>43.13582199953217</v>
+        <v>54.89195528384244</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>35.94337141665129</v>
+        <v>13.84676242588044</v>
       </c>
       <c r="J56" s="2" t="n">
-        <v>0.2287138178739422</v>
+        <v>1.701396182975228</v>
       </c>
       <c r="K56" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L56" s="2" t="n">
         <v>0</v>
@@ -3432,31 +3432,31 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>-2.941315064776461</v>
+        <v>0.3910592841563549</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, dealer_buy_3d, mfi_strong, above_ichimoku_cloud</t>
+          <t>volume_break, market_above_ma60, liquidity_ok, stronger_than_market, kd_golden_cross, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>6121</v>
+        <v>6155</v>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>新普</t>
+          <t>鈞寶</t>
         </is>
       </c>
       <c r="C57" s="2" t="n">
         <v/>
       </c>
       <c r="D57" s="2" t="n">
-        <v>628.2195400059877</v>
+        <v>629.4959232885302</v>
       </c>
       <c r="E57" s="2" t="n">
-        <v>420.5</v>
+        <v>73.2</v>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
@@ -3467,29 +3467,29 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>51.03227255657332</v>
+        <v>43.13582199953217</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>27.22275376749933</v>
+        <v>35.94337141665129</v>
       </c>
       <c r="J57" s="2" t="n">
-        <v>0.8908416609528386</v>
+        <v>0.2287138178739422</v>
       </c>
       <c r="K57" s="2" t="n">
         <v>0</v>
       </c>
       <c r="L57" s="2" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M57" s="2" t="n">
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>0.4387885168904137</v>
+        <v>-2.941315064776461</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, invest_trust_buy_2d, mfi_strong, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending, dealer_buy_3d, mfi_strong, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
@@ -11180,21 +11180,21 @@
     </row>
     <row r="203">
       <c r="A203" s="2" t="n">
-        <v>4569</v>
+        <v>6118</v>
       </c>
       <c r="B203" s="2" t="inlineStr">
         <is>
-          <t>六方科-KY</t>
+          <t>建達</t>
         </is>
       </c>
       <c r="C203" s="2" t="n">
         <v/>
       </c>
       <c r="D203" s="2" t="n">
-        <v>302.9075053542104</v>
+        <v>304.7795295513919</v>
       </c>
       <c r="E203" s="2" t="n">
-        <v>168</v>
+        <v>16.8</v>
       </c>
       <c r="F203" s="2" t="inlineStr">
         <is>
@@ -11205,16 +11205,16 @@
         <v>0</v>
       </c>
       <c r="H203" s="2" t="n">
-        <v>44.35197039970742</v>
+        <v>45.47080288711332</v>
       </c>
       <c r="I203" s="2" t="n">
-        <v>10.84488374904044</v>
+        <v>15.38228193099668</v>
       </c>
       <c r="J203" s="2" t="n">
-        <v>0.2551052167447651</v>
+        <v>0.4450346103415014</v>
       </c>
       <c r="K203" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L203" s="2" t="n">
         <v>0</v>
@@ -11223,31 +11223,31 @@
         <v>-1</v>
       </c>
       <c r="N203" s="2" t="n">
-        <v>-0.7512670034810964</v>
+        <v>0.0147630950408104</v>
       </c>
       <c r="O203" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="2" t="n">
-        <v>4766</v>
+        <v>4569</v>
       </c>
       <c r="B204" s="2" t="inlineStr">
         <is>
-          <t>南寶</t>
+          <t>六方科-KY</t>
         </is>
       </c>
       <c r="C204" s="2" t="n">
         <v/>
       </c>
       <c r="D204" s="2" t="n">
-        <v>300.0170681805484</v>
+        <v>302.9075053542104</v>
       </c>
       <c r="E204" s="2" t="n">
-        <v>339.5</v>
+        <v>168</v>
       </c>
       <c r="F204" s="2" t="inlineStr">
         <is>
@@ -11258,13 +11258,13 @@
         <v>0</v>
       </c>
       <c r="H204" s="2" t="n">
-        <v>39.46019507012367</v>
+        <v>44.35197039970742</v>
       </c>
       <c r="I204" s="2" t="n">
-        <v>14.70084476033016</v>
+        <v>10.84488374904044</v>
       </c>
       <c r="J204" s="2" t="n">
-        <v>0.8748072734315264</v>
+        <v>0.2551052167447651</v>
       </c>
       <c r="K204" s="2" t="n">
         <v>0</v>
@@ -11276,31 +11276,31 @@
         <v>-1</v>
       </c>
       <c r="N204" s="2" t="n">
-        <v>-0.8274155175436628</v>
+        <v>-0.7512670034810964</v>
       </c>
       <c r="O204" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="2" t="n">
-        <v>4749</v>
+        <v>4766</v>
       </c>
       <c r="B205" s="2" t="inlineStr">
         <is>
-          <t>新應材</t>
+          <t>南寶</t>
         </is>
       </c>
       <c r="C205" s="2" t="n">
         <v/>
       </c>
       <c r="D205" s="2" t="n">
-        <v>299.4901212288082</v>
+        <v>300.0170681805484</v>
       </c>
       <c r="E205" s="2" t="n">
-        <v>866</v>
+        <v>339.5</v>
       </c>
       <c r="F205" s="2" t="inlineStr">
         <is>
@@ -11311,13 +11311,13 @@
         <v>0</v>
       </c>
       <c r="H205" s="2" t="n">
-        <v>38.41594582034104</v>
+        <v>39.46019507012367</v>
       </c>
       <c r="I205" s="2" t="n">
-        <v>15.08476122422519</v>
+        <v>14.70084476033016</v>
       </c>
       <c r="J205" s="2" t="n">
-        <v>0.5141350847567634</v>
+        <v>0.8748072734315264</v>
       </c>
       <c r="K205" s="2" t="n">
         <v>0</v>
@@ -11329,7 +11329,7 @@
         <v>-1</v>
       </c>
       <c r="N205" s="2" t="n">
-        <v>-0.6896536427289561</v>
+        <v>-0.8274155175436628</v>
       </c>
       <c r="O205" s="2" t="inlineStr">
         <is>
@@ -11339,21 +11339,21 @@
     </row>
     <row r="206">
       <c r="A206" s="2" t="n">
-        <v>5493</v>
+        <v>4749</v>
       </c>
       <c r="B206" s="2" t="inlineStr">
         <is>
-          <t>三聯</t>
+          <t>新應材</t>
         </is>
       </c>
       <c r="C206" s="2" t="n">
         <v/>
       </c>
       <c r="D206" s="2" t="n">
-        <v>297.3169791208526</v>
+        <v>299.4901212288082</v>
       </c>
       <c r="E206" s="2" t="n">
-        <v>88.8</v>
+        <v>866</v>
       </c>
       <c r="F206" s="2" t="inlineStr">
         <is>
@@ -11364,13 +11364,13 @@
         <v>0</v>
       </c>
       <c r="H206" s="2" t="n">
-        <v>43.82264082381099</v>
+        <v>38.41594582034104</v>
       </c>
       <c r="I206" s="2" t="n">
-        <v>12.6575771778006</v>
+        <v>15.08476122422519</v>
       </c>
       <c r="J206" s="2" t="n">
-        <v>0.3782736683799245</v>
+        <v>0.5141350847567634</v>
       </c>
       <c r="K206" s="2" t="n">
         <v>0</v>
@@ -11382,31 +11382,31 @@
         <v>-1</v>
       </c>
       <c r="N206" s="2" t="n">
-        <v>-0.4119212211238036</v>
+        <v>-0.6896536427289561</v>
       </c>
       <c r="O206" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="2" t="n">
-        <v>4908</v>
+        <v>5493</v>
       </c>
       <c r="B207" s="2" t="inlineStr">
         <is>
-          <t>前鼎</t>
+          <t>三聯</t>
         </is>
       </c>
       <c r="C207" s="2" t="n">
         <v/>
       </c>
       <c r="D207" s="2" t="n">
-        <v>297.0682008883806</v>
+        <v>297.3169791208526</v>
       </c>
       <c r="E207" s="2" t="n">
-        <v>164</v>
+        <v>88.8</v>
       </c>
       <c r="F207" s="2" t="inlineStr">
         <is>
@@ -11417,16 +11417,16 @@
         <v>0</v>
       </c>
       <c r="H207" s="2" t="n">
-        <v>38.12299625897704</v>
+        <v>43.82264082381099</v>
       </c>
       <c r="I207" s="2" t="n">
-        <v>15.65156815142496</v>
+        <v>12.6575771778006</v>
       </c>
       <c r="J207" s="2" t="n">
-        <v>0.5937629711586058</v>
+        <v>0.3782736683799245</v>
       </c>
       <c r="K207" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L207" s="2" t="n">
         <v>0</v>
@@ -11435,31 +11435,31 @@
         <v>-1</v>
       </c>
       <c r="N207" s="2" t="n">
-        <v>-2.272310132552802</v>
+        <v>-0.4119212211238036</v>
       </c>
       <c r="O207" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="2" t="n">
-        <v>6160</v>
+        <v>4908</v>
       </c>
       <c r="B208" s="2" t="inlineStr">
         <is>
-          <t>欣技</t>
+          <t>前鼎</t>
         </is>
       </c>
       <c r="C208" s="2" t="n">
         <v/>
       </c>
       <c r="D208" s="2" t="n">
-        <v>295.9472747077183</v>
+        <v>297.0682008883806</v>
       </c>
       <c r="E208" s="2" t="n">
-        <v>16.45</v>
+        <v>164</v>
       </c>
       <c r="F208" s="2" t="inlineStr">
         <is>
@@ -11470,16 +11470,16 @@
         <v>0</v>
       </c>
       <c r="H208" s="2" t="n">
-        <v>48.22604353199389</v>
+        <v>38.12299625897704</v>
       </c>
       <c r="I208" s="2" t="n">
-        <v>15.48624988224888</v>
+        <v>15.65156815142496</v>
       </c>
       <c r="J208" s="2" t="n">
-        <v>0.3212587975295412</v>
+        <v>0.5937629711586058</v>
       </c>
       <c r="K208" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L208" s="2" t="n">
         <v>0</v>
@@ -11488,31 +11488,31 @@
         <v>-1</v>
       </c>
       <c r="N208" s="2" t="n">
-        <v>-0.0229145721072115</v>
+        <v>-2.272310132552802</v>
       </c>
       <c r="O208" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="2" t="n">
-        <v>4441</v>
+        <v>6160</v>
       </c>
       <c r="B209" s="2" t="inlineStr">
         <is>
-          <t>振大環球</t>
+          <t>欣技</t>
         </is>
       </c>
       <c r="C209" s="2" t="n">
         <v/>
       </c>
       <c r="D209" s="2" t="n">
-        <v>295.7694818552695</v>
+        <v>295.9472747077183</v>
       </c>
       <c r="E209" s="2" t="n">
-        <v>190</v>
+        <v>16.45</v>
       </c>
       <c r="F209" s="2" t="inlineStr">
         <is>
@@ -11523,13 +11523,13 @@
         <v>0</v>
       </c>
       <c r="H209" s="2" t="n">
-        <v>43.19565203222257</v>
+        <v>48.22604353199389</v>
       </c>
       <c r="I209" s="2" t="n">
-        <v>10.23073100744191</v>
+        <v>15.48624988224888</v>
       </c>
       <c r="J209" s="2" t="n">
-        <v>0.5269748961677119</v>
+        <v>0.3212587975295412</v>
       </c>
       <c r="K209" s="2" t="n">
         <v>0</v>
@@ -11541,31 +11541,31 @@
         <v>-1</v>
       </c>
       <c r="N209" s="2" t="n">
-        <v>-0.0183379228354452</v>
+        <v>-0.0229145721072115</v>
       </c>
       <c r="O209" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="2" t="n">
-        <v>4927</v>
+        <v>4441</v>
       </c>
       <c r="B210" s="2" t="inlineStr">
         <is>
-          <t>泰鼎-KY</t>
+          <t>振大環球</t>
         </is>
       </c>
       <c r="C210" s="2" t="n">
         <v/>
       </c>
       <c r="D210" s="2" t="n">
-        <v>295.1088722448619</v>
+        <v>295.7694818552695</v>
       </c>
       <c r="E210" s="2" t="n">
-        <v>40.85</v>
+        <v>190</v>
       </c>
       <c r="F210" s="2" t="inlineStr">
         <is>
@@ -11576,16 +11576,16 @@
         <v>0</v>
       </c>
       <c r="H210" s="2" t="n">
-        <v>32.98711162876012</v>
+        <v>43.19565203222257</v>
       </c>
       <c r="I210" s="2" t="n">
-        <v>14.67295734240476</v>
+        <v>10.23073100744191</v>
       </c>
       <c r="J210" s="2" t="n">
-        <v>0.5670694249202706</v>
+        <v>0.5269748961677119</v>
       </c>
       <c r="K210" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L210" s="2" t="n">
         <v>0</v>
@@ -11594,31 +11594,31 @@
         <v>-1</v>
       </c>
       <c r="N210" s="2" t="n">
-        <v>-0.6573811394869182</v>
+        <v>-0.0183379228354452</v>
       </c>
       <c r="O210" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="2" t="n">
-        <v>6115</v>
+        <v>4927</v>
       </c>
       <c r="B211" s="2" t="inlineStr">
         <is>
-          <t>鎰勝</t>
+          <t>泰鼎-KY</t>
         </is>
       </c>
       <c r="C211" s="2" t="n">
         <v/>
       </c>
       <c r="D211" s="2" t="n">
-        <v>295.0121190764257</v>
+        <v>295.1088722448619</v>
       </c>
       <c r="E211" s="2" t="n">
-        <v>46</v>
+        <v>40.85</v>
       </c>
       <c r="F211" s="2" t="inlineStr">
         <is>
@@ -11629,16 +11629,16 @@
         <v>0</v>
       </c>
       <c r="H211" s="2" t="n">
-        <v>28.99905481585751</v>
+        <v>32.98711162876012</v>
       </c>
       <c r="I211" s="2" t="n">
-        <v>11.87243000552014</v>
+        <v>14.67295734240476</v>
       </c>
       <c r="J211" s="2" t="n">
-        <v>1.784466173498471</v>
+        <v>0.5670694249202706</v>
       </c>
       <c r="K211" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L211" s="2" t="n">
         <v>0</v>
@@ -11647,31 +11647,31 @@
         <v>-1</v>
       </c>
       <c r="N211" s="2" t="n">
-        <v>-0.2027526749396899</v>
+        <v>-0.6573811394869182</v>
       </c>
       <c r="O211" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="2" t="n">
-        <v>5284</v>
+        <v>6115</v>
       </c>
       <c r="B212" s="2" t="inlineStr">
         <is>
-          <t>jpp-KY</t>
+          <t>鎰勝</t>
         </is>
       </c>
       <c r="C212" s="2" t="n">
         <v/>
       </c>
       <c r="D212" s="2" t="n">
-        <v>293.7502424532429</v>
+        <v>295.0121190764257</v>
       </c>
       <c r="E212" s="2" t="n">
-        <v>330</v>
+        <v>46</v>
       </c>
       <c r="F212" s="2" t="inlineStr">
         <is>
@@ -11682,13 +11682,13 @@
         <v>0</v>
       </c>
       <c r="H212" s="2" t="n">
-        <v>35.39337445597386</v>
+        <v>28.99905481585751</v>
       </c>
       <c r="I212" s="2" t="n">
-        <v>16.86858812202756</v>
+        <v>11.87243000552014</v>
       </c>
       <c r="J212" s="2" t="n">
-        <v>0.5909194086228496</v>
+        <v>1.784466173498471</v>
       </c>
       <c r="K212" s="2" t="n">
         <v>0</v>
@@ -11700,31 +11700,31 @@
         <v>-1</v>
       </c>
       <c r="N212" s="2" t="n">
-        <v>-5.297048187949795</v>
+        <v>-0.2027526749396899</v>
       </c>
       <c r="O212" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>ema60_gt_ema120, volume_break, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="2" t="n">
-        <v>4906</v>
+        <v>5284</v>
       </c>
       <c r="B213" s="2" t="inlineStr">
         <is>
-          <t>正文</t>
+          <t>jpp-KY</t>
         </is>
       </c>
       <c r="C213" s="2" t="n">
         <v/>
       </c>
       <c r="D213" s="2" t="n">
-        <v>293.7196725846934</v>
+        <v>293.7502424532429</v>
       </c>
       <c r="E213" s="2" t="n">
-        <v>39.9</v>
+        <v>330</v>
       </c>
       <c r="F213" s="2" t="inlineStr">
         <is>
@@ -11735,13 +11735,13 @@
         <v>0</v>
       </c>
       <c r="H213" s="2" t="n">
-        <v>42.54640859701222</v>
+        <v>35.39337445597386</v>
       </c>
       <c r="I213" s="2" t="n">
-        <v>15.27255548104496</v>
+        <v>16.86858812202756</v>
       </c>
       <c r="J213" s="2" t="n">
-        <v>0.4152784620076702</v>
+        <v>0.5909194086228496</v>
       </c>
       <c r="K213" s="2" t="n">
         <v>0</v>
@@ -11753,31 +11753,31 @@
         <v>-1</v>
       </c>
       <c r="N213" s="2" t="n">
-        <v>-0.4987165533848428</v>
+        <v>-5.297048187949795</v>
       </c>
       <c r="O213" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="2" t="n">
-        <v>4979</v>
+        <v>4906</v>
       </c>
       <c r="B214" s="2" t="inlineStr">
         <is>
-          <t>華星光</t>
+          <t>正文</t>
         </is>
       </c>
       <c r="C214" s="2" t="n">
         <v/>
       </c>
       <c r="D214" s="2" t="n">
-        <v>279.9811611625873</v>
+        <v>293.7196725846934</v>
       </c>
       <c r="E214" s="2" t="n">
-        <v>432.5</v>
+        <v>39.9</v>
       </c>
       <c r="F214" s="2" t="inlineStr">
         <is>
@@ -11788,13 +11788,13 @@
         <v>0</v>
       </c>
       <c r="H214" s="2" t="n">
-        <v>37.46788183948913</v>
+        <v>42.54640859701222</v>
       </c>
       <c r="I214" s="2" t="n">
-        <v>14.6584267850354</v>
+        <v>15.27255548104496</v>
       </c>
       <c r="J214" s="2" t="n">
-        <v>0.5133019543243857</v>
+        <v>0.4152784620076702</v>
       </c>
       <c r="K214" s="2" t="n">
         <v>0</v>
@@ -11806,31 +11806,31 @@
         <v>-1</v>
       </c>
       <c r="N214" s="2" t="n">
-        <v>-3.802555078672937</v>
+        <v>-0.4987165533848428</v>
       </c>
       <c r="O214" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="2" t="n">
-        <v>4935</v>
+        <v>4979</v>
       </c>
       <c r="B215" s="2" t="inlineStr">
         <is>
-          <t>茂林-KY</t>
+          <t>華星光</t>
         </is>
       </c>
       <c r="C215" s="2" t="n">
         <v/>
       </c>
       <c r="D215" s="2" t="n">
-        <v>279.1970821055019</v>
+        <v>279.9811611625873</v>
       </c>
       <c r="E215" s="2" t="n">
-        <v>36.15</v>
+        <v>432.5</v>
       </c>
       <c r="F215" s="2" t="inlineStr">
         <is>
@@ -11841,13 +11841,13 @@
         <v>0</v>
       </c>
       <c r="H215" s="2" t="n">
-        <v>41.51680575810931</v>
+        <v>37.46788183948913</v>
       </c>
       <c r="I215" s="2" t="n">
-        <v>14.37677731443604</v>
+        <v>14.6584267850354</v>
       </c>
       <c r="J215" s="2" t="n">
-        <v>0.5522513970281732</v>
+        <v>0.5133019543243857</v>
       </c>
       <c r="K215" s="2" t="n">
         <v>0</v>
@@ -11859,31 +11859,31 @@
         <v>-1</v>
       </c>
       <c r="N215" s="2" t="n">
-        <v>-0.2397104843468199</v>
+        <v>-3.802555078672937</v>
       </c>
       <c r="O215" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="2" t="n">
-        <v>5244</v>
+        <v>4935</v>
       </c>
       <c r="B216" s="2" t="inlineStr">
         <is>
-          <t>弘凱</t>
+          <t>茂林-KY</t>
         </is>
       </c>
       <c r="C216" s="2" t="n">
         <v/>
       </c>
       <c r="D216" s="2" t="n">
-        <v>278.3572224260511</v>
+        <v>279.1970821055019</v>
       </c>
       <c r="E216" s="2" t="n">
-        <v>34.1</v>
+        <v>36.15</v>
       </c>
       <c r="F216" s="2" t="inlineStr">
         <is>
@@ -11894,16 +11894,16 @@
         <v>0</v>
       </c>
       <c r="H216" s="2" t="n">
-        <v>30.73414277687705</v>
+        <v>41.51680575810931</v>
       </c>
       <c r="I216" s="2" t="n">
-        <v>19.40876087724228</v>
+        <v>14.37677731443604</v>
       </c>
       <c r="J216" s="2" t="n">
-        <v>0.8161669547188597</v>
+        <v>0.5522513970281732</v>
       </c>
       <c r="K216" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L216" s="2" t="n">
         <v>0</v>
@@ -11912,31 +11912,31 @@
         <v>-1</v>
       </c>
       <c r="N216" s="2" t="n">
-        <v>-0.1874712137610277</v>
+        <v>-0.2397104843468199</v>
       </c>
       <c r="O216" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="2" t="n">
-        <v>5355</v>
+        <v>5244</v>
       </c>
       <c r="B217" s="2" t="inlineStr">
         <is>
-          <t>佳總</t>
+          <t>弘凱</t>
         </is>
       </c>
       <c r="C217" s="2" t="n">
         <v/>
       </c>
       <c r="D217" s="2" t="n">
-        <v>278.0838016630031</v>
+        <v>278.3572224260511</v>
       </c>
       <c r="E217" s="2" t="n">
-        <v>6.15</v>
+        <v>34.1</v>
       </c>
       <c r="F217" s="2" t="inlineStr">
         <is>
@@ -11947,16 +11947,16 @@
         <v>0</v>
       </c>
       <c r="H217" s="2" t="n">
-        <v>42.27261439055491</v>
+        <v>30.73414277687705</v>
       </c>
       <c r="I217" s="2" t="n">
-        <v>11.46893304418927</v>
+        <v>19.40876087724228</v>
       </c>
       <c r="J217" s="2" t="n">
-        <v>0.1792063924452919</v>
+        <v>0.8161669547188597</v>
       </c>
       <c r="K217" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L217" s="2" t="n">
         <v>0</v>
@@ -11965,31 +11965,31 @@
         <v>-1</v>
       </c>
       <c r="N217" s="2" t="n">
-        <v>-0.0283885377492316</v>
+        <v>-0.1874712137610277</v>
       </c>
       <c r="O217" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="2" t="n">
-        <v>5223</v>
+        <v>5355</v>
       </c>
       <c r="B218" s="2" t="inlineStr">
         <is>
-          <t>安力-KY</t>
+          <t>佳總</t>
         </is>
       </c>
       <c r="C218" s="2" t="n">
         <v/>
       </c>
       <c r="D218" s="2" t="n">
-        <v>269.2621382503258</v>
+        <v>278.0838016630031</v>
       </c>
       <c r="E218" s="2" t="n">
-        <v>25.1</v>
+        <v>6.15</v>
       </c>
       <c r="F218" s="2" t="inlineStr">
         <is>
@@ -12000,13 +12000,13 @@
         <v>0</v>
       </c>
       <c r="H218" s="2" t="n">
-        <v>47.24135543562591</v>
+        <v>42.27261439055491</v>
       </c>
       <c r="I218" s="2" t="n">
-        <v>11.8640824707857</v>
+        <v>11.46893304418927</v>
       </c>
       <c r="J218" s="2" t="n">
-        <v>0.6699769822082604</v>
+        <v>0.1792063924452919</v>
       </c>
       <c r="K218" s="2" t="n">
         <v>0</v>
@@ -12018,31 +12018,31 @@
         <v>-1</v>
       </c>
       <c r="N218" s="2" t="n">
-        <v>-0.0306412873125715</v>
+        <v>-0.0283885377492316</v>
       </c>
       <c r="O218" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="2" t="n">
-        <v>5907</v>
+        <v>5223</v>
       </c>
       <c r="B219" s="2" t="inlineStr">
         <is>
-          <t>大洋-KY</t>
+          <t>安力-KY</t>
         </is>
       </c>
       <c r="C219" s="2" t="n">
         <v/>
       </c>
       <c r="D219" s="2" t="n">
-        <v>269.2482495846094</v>
+        <v>269.2621382503258</v>
       </c>
       <c r="E219" s="2" t="n">
-        <v>5</v>
+        <v>25.1</v>
       </c>
       <c r="F219" s="2" t="inlineStr">
         <is>
@@ -12053,13 +12053,13 @@
         <v>0</v>
       </c>
       <c r="H219" s="2" t="n">
-        <v>47.79668669007309</v>
+        <v>47.24135543562591</v>
       </c>
       <c r="I219" s="2" t="n">
-        <v>15.76889386142467</v>
+        <v>11.8640824707857</v>
       </c>
       <c r="J219" s="2" t="n">
-        <v>0.6145006401614048</v>
+        <v>0.6699769822082604</v>
       </c>
       <c r="K219" s="2" t="n">
         <v>0</v>
@@ -12071,31 +12071,31 @@
         <v>-1</v>
       </c>
       <c r="N219" s="2" t="n">
-        <v>0.0161476811107272</v>
+        <v>-0.0306412873125715</v>
       </c>
       <c r="O219" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="2" t="n">
-        <v>6126</v>
+        <v>5907</v>
       </c>
       <c r="B220" s="2" t="inlineStr">
         <is>
-          <t>信音</t>
+          <t>大洋-KY</t>
         </is>
       </c>
       <c r="C220" s="2" t="n">
         <v/>
       </c>
       <c r="D220" s="2" t="n">
-        <v>267.3416794752319</v>
+        <v>269.2482495846094</v>
       </c>
       <c r="E220" s="2" t="n">
-        <v>35.1</v>
+        <v>5</v>
       </c>
       <c r="F220" s="2" t="inlineStr">
         <is>
@@ -12106,13 +12106,13 @@
         <v>0</v>
       </c>
       <c r="H220" s="2" t="n">
-        <v>43.61578752793271</v>
+        <v>47.79668669007309</v>
       </c>
       <c r="I220" s="2" t="n">
-        <v>19.76910082572275</v>
+        <v>15.76889386142467</v>
       </c>
       <c r="J220" s="2" t="n">
-        <v>0.4120017597494858</v>
+        <v>0.6145006401614048</v>
       </c>
       <c r="K220" s="2" t="n">
         <v>0</v>
@@ -12124,31 +12124,31 @@
         <v>-1</v>
       </c>
       <c r="N220" s="2" t="n">
-        <v>-0.4823696551610847</v>
+        <v>0.0161476811107272</v>
       </c>
       <c r="O220" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="2" t="n">
-        <v>5533</v>
+        <v>6126</v>
       </c>
       <c r="B221" s="2" t="inlineStr">
         <is>
-          <t>皇鼎</t>
+          <t>信音</t>
         </is>
       </c>
       <c r="C221" s="2" t="n">
         <v/>
       </c>
       <c r="D221" s="2" t="n">
-        <v>255.9211715042628</v>
+        <v>267.3416794752319</v>
       </c>
       <c r="E221" s="2" t="n">
-        <v>13.55</v>
+        <v>35.1</v>
       </c>
       <c r="F221" s="2" t="inlineStr">
         <is>
@@ -12159,13 +12159,13 @@
         <v>0</v>
       </c>
       <c r="H221" s="2" t="n">
-        <v>31.52991060471417</v>
+        <v>43.61578752793271</v>
       </c>
       <c r="I221" s="2" t="n">
-        <v>18.03919083634613</v>
+        <v>19.76910082572275</v>
       </c>
       <c r="J221" s="2" t="n">
-        <v>1.506808682151609</v>
+        <v>0.4120017597494858</v>
       </c>
       <c r="K221" s="2" t="n">
         <v>0</v>
@@ -12177,31 +12177,31 @@
         <v>-1</v>
       </c>
       <c r="N221" s="2" t="n">
-        <v>-0.0167022838843169</v>
+        <v>-0.4823696551610847</v>
       </c>
       <c r="O221" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="2" t="n">
-        <v>5215</v>
+        <v>5533</v>
       </c>
       <c r="B222" s="2" t="inlineStr">
         <is>
-          <t>科嘉-KY</t>
+          <t>皇鼎</t>
         </is>
       </c>
       <c r="C222" s="2" t="n">
         <v/>
       </c>
       <c r="D222" s="2" t="n">
-        <v>252.5216171842064</v>
+        <v>255.9211715042628</v>
       </c>
       <c r="E222" s="2" t="n">
-        <v>42.05</v>
+        <v>13.55</v>
       </c>
       <c r="F222" s="2" t="inlineStr">
         <is>
@@ -12212,13 +12212,13 @@
         <v>0</v>
       </c>
       <c r="H222" s="2" t="n">
-        <v>40.44961131382579</v>
+        <v>31.52991060471417</v>
       </c>
       <c r="I222" s="2" t="n">
-        <v>17.79510544211668</v>
+        <v>18.03919083634613</v>
       </c>
       <c r="J222" s="2" t="n">
-        <v>0.6320208568142058</v>
+        <v>1.506808682151609</v>
       </c>
       <c r="K222" s="2" t="n">
         <v>0</v>
@@ -12230,31 +12230,31 @@
         <v>-1</v>
       </c>
       <c r="N222" s="2" t="n">
-        <v>-0.1625597039914724</v>
+        <v>-0.0167022838843169</v>
       </c>
       <c r="O222" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>volume_break, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="2" t="n">
-        <v>5251</v>
+        <v>5215</v>
       </c>
       <c r="B223" s="2" t="inlineStr">
         <is>
-          <t>天鉞電</t>
+          <t>科嘉-KY</t>
         </is>
       </c>
       <c r="C223" s="2" t="n">
         <v/>
       </c>
       <c r="D223" s="2" t="n">
-        <v>251.3458342952489</v>
+        <v>252.5216171842064</v>
       </c>
       <c r="E223" s="2" t="n">
-        <v>29.4</v>
+        <v>42.05</v>
       </c>
       <c r="F223" s="2" t="inlineStr">
         <is>
@@ -12265,13 +12265,13 @@
         <v>0</v>
       </c>
       <c r="H223" s="2" t="n">
-        <v>44.51691164762632</v>
+        <v>40.44961131382579</v>
       </c>
       <c r="I223" s="2" t="n">
-        <v>33.97967568033089</v>
+        <v>17.79510544211668</v>
       </c>
       <c r="J223" s="2" t="n">
-        <v>0.218075517245245</v>
+        <v>0.6320208568142058</v>
       </c>
       <c r="K223" s="2" t="n">
         <v>0</v>
@@ -12283,31 +12283,31 @@
         <v>-1</v>
       </c>
       <c r="N223" s="2" t="n">
-        <v>-0.3081314926700571</v>
+        <v>-0.1625597039914724</v>
       </c>
       <c r="O223" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="2" t="n">
-        <v>4999</v>
+        <v>5251</v>
       </c>
       <c r="B224" s="2" t="inlineStr">
         <is>
-          <t>鑫禾</t>
+          <t>天鉞電</t>
         </is>
       </c>
       <c r="C224" s="2" t="n">
         <v/>
       </c>
       <c r="D224" s="2" t="n">
-        <v>247.5085659534315</v>
+        <v>251.3458342952489</v>
       </c>
       <c r="E224" s="2" t="n">
-        <v>20.05</v>
+        <v>29.4</v>
       </c>
       <c r="F224" s="2" t="inlineStr">
         <is>
@@ -12318,13 +12318,13 @@
         <v>0</v>
       </c>
       <c r="H224" s="2" t="n">
-        <v>43.34636265348431</v>
+        <v>44.51691164762632</v>
       </c>
       <c r="I224" s="2" t="n">
-        <v>13.45189436139593</v>
+        <v>33.97967568033089</v>
       </c>
       <c r="J224" s="2" t="n">
-        <v>0.4908520665582417</v>
+        <v>0.218075517245245</v>
       </c>
       <c r="K224" s="2" t="n">
         <v>0</v>
@@ -12336,31 +12336,31 @@
         <v>-1</v>
       </c>
       <c r="N224" s="2" t="n">
-        <v>-0.0121728982650053</v>
+        <v>-0.3081314926700571</v>
       </c>
       <c r="O224" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="2" t="n">
-        <v>4588</v>
+        <v>4999</v>
       </c>
       <c r="B225" s="2" t="inlineStr">
         <is>
-          <t>玖鼎電力</t>
+          <t>鑫禾</t>
         </is>
       </c>
       <c r="C225" s="2" t="n">
         <v/>
       </c>
       <c r="D225" s="2" t="n">
-        <v>243.5567806250405</v>
+        <v>247.5085659534315</v>
       </c>
       <c r="E225" s="2" t="n">
-        <v>57.5</v>
+        <v>20.05</v>
       </c>
       <c r="F225" s="2" t="inlineStr">
         <is>
@@ -12371,13 +12371,13 @@
         <v>0</v>
       </c>
       <c r="H225" s="2" t="n">
-        <v>45.47873697416233</v>
+        <v>43.34636265348431</v>
       </c>
       <c r="I225" s="2" t="n">
-        <v>16.9470277194014</v>
+        <v>13.45189436139593</v>
       </c>
       <c r="J225" s="2" t="n">
-        <v>0.3763262554525466</v>
+        <v>0.4908520665582417</v>
       </c>
       <c r="K225" s="2" t="n">
         <v>0</v>
@@ -12389,31 +12389,31 @@
         <v>-1</v>
       </c>
       <c r="N225" s="2" t="n">
-        <v>-0.214344634265602</v>
+        <v>-0.0121728982650053</v>
       </c>
       <c r="O225" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="2" t="n">
-        <v>4943</v>
+        <v>4588</v>
       </c>
       <c r="B226" s="2" t="inlineStr">
         <is>
-          <t>康控-KY</t>
+          <t>玖鼎電力</t>
         </is>
       </c>
       <c r="C226" s="2" t="n">
         <v/>
       </c>
       <c r="D226" s="2" t="n">
-        <v>210.6325198201673</v>
+        <v>243.5567806250405</v>
       </c>
       <c r="E226" s="2" t="n">
-        <v>8.6</v>
+        <v>57.5</v>
       </c>
       <c r="F226" s="2" t="inlineStr">
         <is>
@@ -12424,13 +12424,13 @@
         <v>0</v>
       </c>
       <c r="H226" s="2" t="n">
-        <v>39.36809894888794</v>
+        <v>45.47873697416233</v>
       </c>
       <c r="I226" s="2" t="n">
-        <v>12.1674077379116</v>
+        <v>16.9470277194014</v>
       </c>
       <c r="J226" s="2" t="n">
-        <v>0.1303036418477045</v>
+        <v>0.3763262554525466</v>
       </c>
       <c r="K226" s="2" t="n">
         <v>0</v>
@@ -12442,31 +12442,31 @@
         <v>-1</v>
       </c>
       <c r="N226" s="2" t="n">
-        <v>-0.0398539638634945</v>
+        <v>-0.214344634265602</v>
       </c>
       <c r="O226" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="2" t="n">
-        <v>4909</v>
+        <v>6123</v>
       </c>
       <c r="B227" s="2" t="inlineStr">
         <is>
-          <t>新復興</t>
+          <t>上奇</t>
         </is>
       </c>
       <c r="C227" s="2" t="n">
         <v/>
       </c>
       <c r="D227" s="2" t="n">
-        <v>205.5031391550787</v>
+        <v>242.8371222838319</v>
       </c>
       <c r="E227" s="2" t="n">
-        <v>42.1</v>
+        <v>42</v>
       </c>
       <c r="F227" s="2" t="inlineStr">
         <is>
@@ -12477,13 +12477,13 @@
         <v>0</v>
       </c>
       <c r="H227" s="2" t="n">
-        <v>29.75377787253753</v>
+        <v>39.81693161364736</v>
       </c>
       <c r="I227" s="2" t="n">
-        <v>32.0785781468538</v>
+        <v>16.2684341224688</v>
       </c>
       <c r="J227" s="2" t="n">
-        <v>0.5982766258543352</v>
+        <v>0.4197489275776593</v>
       </c>
       <c r="K227" s="2" t="n">
         <v>1</v>
@@ -12495,31 +12495,31 @@
         <v>-1</v>
       </c>
       <c r="N227" s="2" t="n">
-        <v>-0.1770602805793091</v>
+        <v>-0.0048265410947612</v>
       </c>
       <c r="O227" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="2" t="n">
-        <v>4977</v>
+        <v>4943</v>
       </c>
       <c r="B228" s="2" t="inlineStr">
         <is>
-          <t>眾達-KY</t>
+          <t>康控-KY</t>
         </is>
       </c>
       <c r="C228" s="2" t="n">
         <v/>
       </c>
       <c r="D228" s="2" t="n">
-        <v>204.6035442325117</v>
+        <v>210.6325198201673</v>
       </c>
       <c r="E228" s="2" t="n">
-        <v>152.5</v>
+        <v>8.6</v>
       </c>
       <c r="F228" s="2" t="inlineStr">
         <is>
@@ -12530,13 +12530,13 @@
         <v>0</v>
       </c>
       <c r="H228" s="2" t="n">
-        <v>37.95345628912644</v>
+        <v>39.36809894888794</v>
       </c>
       <c r="I228" s="2" t="n">
-        <v>11.43809731641805</v>
+        <v>12.1674077379116</v>
       </c>
       <c r="J228" s="2" t="n">
-        <v>0.5166270747649936</v>
+        <v>0.1303036418477045</v>
       </c>
       <c r="K228" s="2" t="n">
         <v>0</v>
@@ -12548,31 +12548,31 @@
         <v>-1</v>
       </c>
       <c r="N228" s="2" t="n">
-        <v>-1.192898054768346</v>
+        <v>-0.0398539638634945</v>
       </c>
       <c r="O228" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="2" t="n">
-        <v>4729</v>
+        <v>4909</v>
       </c>
       <c r="B229" s="2" t="inlineStr">
         <is>
-          <t>熒茂</t>
+          <t>新復興</t>
         </is>
       </c>
       <c r="C229" s="2" t="n">
         <v/>
       </c>
       <c r="D229" s="2" t="n">
-        <v>199.5085187436612</v>
+        <v>205.5031391550787</v>
       </c>
       <c r="E229" s="2" t="n">
-        <v>21.4</v>
+        <v>42.1</v>
       </c>
       <c r="F229" s="2" t="inlineStr">
         <is>
@@ -12583,16 +12583,16 @@
         <v>0</v>
       </c>
       <c r="H229" s="2" t="n">
-        <v>43.95043295934696</v>
+        <v>29.75377787253753</v>
       </c>
       <c r="I229" s="2" t="n">
-        <v>14.9702916573282</v>
+        <v>32.0785781468538</v>
       </c>
       <c r="J229" s="2" t="n">
-        <v>0.4359799038798103</v>
+        <v>0.5982766258543352</v>
       </c>
       <c r="K229" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L229" s="2" t="n">
         <v>0</v>
@@ -12601,31 +12601,31 @@
         <v>-1</v>
       </c>
       <c r="N229" s="2" t="n">
-        <v>-0.1052787399476526</v>
+        <v>-0.1770602805793091</v>
       </c>
       <c r="O229" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="2" t="n">
-        <v>5906</v>
+        <v>4977</v>
       </c>
       <c r="B230" s="2" t="inlineStr">
         <is>
-          <t>台南-KY</t>
+          <t>眾達-KY</t>
         </is>
       </c>
       <c r="C230" s="2" t="n">
         <v/>
       </c>
       <c r="D230" s="2" t="n">
-        <v>197.3956783057093</v>
+        <v>204.6035442325117</v>
       </c>
       <c r="E230" s="2" t="n">
-        <v>36.8</v>
+        <v>152.5</v>
       </c>
       <c r="F230" s="2" t="inlineStr">
         <is>
@@ -12636,16 +12636,16 @@
         <v>0</v>
       </c>
       <c r="H230" s="2" t="n">
-        <v>52.02983912912743</v>
+        <v>37.95345628912644</v>
       </c>
       <c r="I230" s="2" t="n">
-        <v>6.037410515784707</v>
+        <v>11.43809731641805</v>
       </c>
       <c r="J230" s="2" t="n">
-        <v>0.0351205888750885</v>
+        <v>0.5166270747649936</v>
       </c>
       <c r="K230" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L230" s="2" t="n">
         <v>0</v>
@@ -12654,31 +12654,31 @@
         <v>-1</v>
       </c>
       <c r="N230" s="2" t="n">
-        <v>0.7802878080530972</v>
+        <v>-1.192898054768346</v>
       </c>
       <c r="O230" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="2" t="n">
-        <v>4905</v>
+        <v>4729</v>
       </c>
       <c r="B231" s="2" t="inlineStr">
         <is>
-          <t>台聯電</t>
+          <t>熒茂</t>
         </is>
       </c>
       <c r="C231" s="2" t="n">
         <v/>
       </c>
       <c r="D231" s="2" t="n">
-        <v>191.7539477623564</v>
+        <v>199.5085187436612</v>
       </c>
       <c r="E231" s="2" t="n">
-        <v>0</v>
+        <v>21.4</v>
       </c>
       <c r="F231" s="2" t="inlineStr">
         <is>
@@ -12689,13 +12689,13 @@
         <v>0</v>
       </c>
       <c r="H231" s="2" t="n">
-        <v>29.1688390277304</v>
+        <v>43.95043295934696</v>
       </c>
       <c r="I231" s="2" t="n">
-        <v>18.34198705604091</v>
+        <v>14.9702916573282</v>
       </c>
       <c r="J231" s="2" t="n">
-        <v>0.008683570684265301</v>
+        <v>0.4359799038798103</v>
       </c>
       <c r="K231" s="2" t="n">
         <v>0</v>
@@ -12707,7 +12707,7 @@
         <v>-1</v>
       </c>
       <c r="N231" s="2" t="n">
-        <v>-3.182526221478449</v>
+        <v>-0.1052787399476526</v>
       </c>
       <c r="O231" s="2" t="inlineStr">
         <is>
@@ -12717,21 +12717,21 @@
     </row>
     <row r="232">
       <c r="A232" s="2" t="n">
-        <v>5465</v>
+        <v>5906</v>
       </c>
       <c r="B232" s="2" t="inlineStr">
         <is>
-          <t>富驊</t>
+          <t>台南-KY</t>
         </is>
       </c>
       <c r="C232" s="2" t="n">
         <v/>
       </c>
       <c r="D232" s="2" t="n">
-        <v>189.4271178827195</v>
+        <v>197.3956783057093</v>
       </c>
       <c r="E232" s="2" t="n">
-        <v>24.9</v>
+        <v>36.8</v>
       </c>
       <c r="F232" s="2" t="inlineStr">
         <is>
@@ -12742,16 +12742,16 @@
         <v>0</v>
       </c>
       <c r="H232" s="2" t="n">
-        <v>42.2943655563449</v>
+        <v>52.02983912912743</v>
       </c>
       <c r="I232" s="2" t="n">
-        <v>13.40399159786386</v>
+        <v>6.037410515784707</v>
       </c>
       <c r="J232" s="2" t="n">
-        <v>0.7003750155767251</v>
+        <v>0.0351205888750885</v>
       </c>
       <c r="K232" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L232" s="2" t="n">
         <v>0</v>
@@ -12760,31 +12760,31 @@
         <v>-1</v>
       </c>
       <c r="N232" s="2" t="n">
-        <v>-0.0398972422383372</v>
+        <v>0.7802878080530972</v>
       </c>
       <c r="O232" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="2" t="n">
-        <v>5315</v>
+        <v>4905</v>
       </c>
       <c r="B233" s="2" t="inlineStr">
         <is>
-          <t>光聯</t>
+          <t>台聯電</t>
         </is>
       </c>
       <c r="C233" s="2" t="n">
         <v/>
       </c>
       <c r="D233" s="2" t="n">
-        <v>180.648487082768</v>
+        <v>191.7539477623564</v>
       </c>
       <c r="E233" s="2" t="n">
-        <v>20.25</v>
+        <v>0</v>
       </c>
       <c r="F233" s="2" t="inlineStr">
         <is>
@@ -12795,16 +12795,16 @@
         <v>0</v>
       </c>
       <c r="H233" s="2" t="n">
-        <v>27.48640193588798</v>
+        <v>29.1688390277304</v>
       </c>
       <c r="I233" s="2" t="n">
-        <v>23.57996354094234</v>
+        <v>18.34198705604091</v>
       </c>
       <c r="J233" s="2" t="n">
-        <v>1.259405918327718</v>
+        <v>0.008683570684265301</v>
       </c>
       <c r="K233" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L233" s="2" t="n">
         <v>0</v>
@@ -12813,31 +12813,31 @@
         <v>-1</v>
       </c>
       <c r="N233" s="2" t="n">
-        <v>-0.335481178521565</v>
+        <v>-3.182526221478449</v>
       </c>
       <c r="O233" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" s="2" t="n">
-        <v>4933</v>
+        <v>5465</v>
       </c>
       <c r="B234" s="2" t="inlineStr">
         <is>
-          <t>友輝</t>
+          <t>富驊</t>
         </is>
       </c>
       <c r="C234" s="2" t="n">
         <v/>
       </c>
       <c r="D234" s="2" t="n">
-        <v>175.6873901105331</v>
+        <v>189.4271178827195</v>
       </c>
       <c r="E234" s="2" t="n">
-        <v>62.6</v>
+        <v>24.9</v>
       </c>
       <c r="F234" s="2" t="inlineStr">
         <is>
@@ -12848,13 +12848,13 @@
         <v>0</v>
       </c>
       <c r="H234" s="2" t="n">
-        <v>34.84321428405289</v>
+        <v>42.2943655563449</v>
       </c>
       <c r="I234" s="2" t="n">
-        <v>12.42311953808553</v>
+        <v>13.40399159786386</v>
       </c>
       <c r="J234" s="2" t="n">
-        <v>1.236613639724996</v>
+        <v>0.7003750155767251</v>
       </c>
       <c r="K234" s="2" t="n">
         <v>0</v>
@@ -12866,31 +12866,31 @@
         <v>-1</v>
       </c>
       <c r="N234" s="2" t="n">
-        <v>-0.2800619343831874</v>
+        <v>-0.0398972422383372</v>
       </c>
       <c r="O234" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, stronger_than_market</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" s="2" t="n">
-        <v>4562</v>
+        <v>5315</v>
       </c>
       <c r="B235" s="2" t="inlineStr">
         <is>
-          <t>穎漢</t>
+          <t>光聯</t>
         </is>
       </c>
       <c r="C235" s="2" t="n">
         <v/>
       </c>
       <c r="D235" s="2" t="n">
-        <v>170.698455264772</v>
+        <v>180.648487082768</v>
       </c>
       <c r="E235" s="2" t="n">
-        <v>34</v>
+        <v>20.25</v>
       </c>
       <c r="F235" s="2" t="inlineStr">
         <is>
@@ -12901,16 +12901,16 @@
         <v>0</v>
       </c>
       <c r="H235" s="2" t="n">
-        <v>42.6660634084714</v>
+        <v>27.48640193588798</v>
       </c>
       <c r="I235" s="2" t="n">
-        <v>13.60222565427213</v>
+        <v>23.57996354094234</v>
       </c>
       <c r="J235" s="2" t="n">
-        <v>0.6726528032138619</v>
+        <v>1.259405918327718</v>
       </c>
       <c r="K235" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L235" s="2" t="n">
         <v>0</v>
@@ -12919,31 +12919,31 @@
         <v>-1</v>
       </c>
       <c r="N235" s="2" t="n">
-        <v>0.0479763214702096</v>
+        <v>-0.335481178521565</v>
       </c>
       <c r="O235" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" s="2" t="n">
-        <v>6118</v>
+        <v>4933</v>
       </c>
       <c r="B236" s="2" t="inlineStr">
         <is>
-          <t>建達</t>
+          <t>友輝</t>
         </is>
       </c>
       <c r="C236" s="2" t="n">
         <v/>
       </c>
       <c r="D236" s="2" t="n">
-        <v>164.7795295513918</v>
+        <v>175.6873901105331</v>
       </c>
       <c r="E236" s="2" t="n">
-        <v>16.8</v>
+        <v>62.6</v>
       </c>
       <c r="F236" s="2" t="inlineStr">
         <is>
@@ -12954,16 +12954,16 @@
         <v>0</v>
       </c>
       <c r="H236" s="2" t="n">
-        <v>45.47080297044787</v>
+        <v>34.84321428405289</v>
       </c>
       <c r="I236" s="2" t="n">
-        <v>15.38228193078404</v>
+        <v>12.42311953808553</v>
       </c>
       <c r="J236" s="2" t="n">
-        <v>0.4450346103415014</v>
+        <v>1.236613639724996</v>
       </c>
       <c r="K236" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L236" s="2" t="n">
         <v>0</v>
@@ -12972,31 +12972,31 @@
         <v>-1</v>
       </c>
       <c r="N236" s="2" t="n">
-        <v>0.0147630950408104</v>
+        <v>-0.2800619343831874</v>
       </c>
       <c r="O236" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" s="2" t="n">
-        <v>6123</v>
+        <v>4562</v>
       </c>
       <c r="B237" s="2" t="inlineStr">
         <is>
-          <t>上奇</t>
+          <t>穎漢</t>
         </is>
       </c>
       <c r="C237" s="2" t="n">
         <v/>
       </c>
       <c r="D237" s="2" t="n">
-        <v>102.8371222838319</v>
+        <v>170.698455264772</v>
       </c>
       <c r="E237" s="2" t="n">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="F237" s="2" t="inlineStr">
         <is>
@@ -13007,16 +13007,16 @@
         <v>0</v>
       </c>
       <c r="H237" s="2" t="n">
-        <v>39.81693151225343</v>
+        <v>42.6660634084714</v>
       </c>
       <c r="I237" s="2" t="n">
-        <v>16.26843409214966</v>
+        <v>13.60222565427213</v>
       </c>
       <c r="J237" s="2" t="n">
-        <v>0.4197489275776593</v>
+        <v>0.6726528032138619</v>
       </c>
       <c r="K237" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L237" s="2" t="n">
         <v>0</v>
@@ -13025,11 +13025,11 @@
         <v>-1</v>
       </c>
       <c r="N237" s="2" t="n">
-        <v>-0.0048265409993495</v>
+        <v>0.0479763214702096</v>
       </c>
       <c r="O237" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>

</xml_diff>